<commit_message>
apply rules for categories / improve underlying logic
</commit_message>
<xml_diff>
--- a/data/test.xlsx
+++ b/data/test.xlsx
@@ -8,9 +8,8 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/taulo/GolandProjects/budgetpipe/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA1A6F2C-5E17-984A-B700-7CE95F030DC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14740" yWindow="5360" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14540" yWindow="8820" windowWidth="28800" windowHeight="17400"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -245,7 +244,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
   <si>
     <t>Januar</t>
   </si>
@@ -377,55 +376,65 @@
   </si>
   <si>
     <t>Hello Worlsssd</t>
+  </si>
+  <si>
+    <t>Udgifter</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;kr.&quot;"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri (Body)"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri (Body)"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Tahoma"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Tahoma"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color rgb="FF000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <i val="1"/>
+      <color theme="1"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -437,7 +446,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -455,13 +464,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.5999938962981048"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor theme="9" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -473,7 +482,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="7" tint="0.3999755851924192"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -708,61 +717,61 @@
   </cellStyleXfs>
   <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="20" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="6" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="7" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="10" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="12" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="13" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="14" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="16" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="5" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="8" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="17" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="15" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="true" applyFill="true"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="5" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="12" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="18" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="13" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="20" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="11" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="19" xfId="0" applyFont="true" applyFill="true" applyBorder="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -775,7 +784,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1143,15 +1152,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AC366279-0C22-F146-A0C6-D2A0D14030D6}">
   <dimension ref="A1:S31"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="14" max="14" width="19" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col bestFit="true" customWidth="true" max="1" min="1" width="27"/>
+    <col bestFit="true" customWidth="true" max="11" min="9" width="11.6640625"/>
+    <col bestFit="true" customWidth="true" max="14" min="14" width="19"/>
+    <col bestFit="true" customWidth="true" max="15" min="15" width="14.6640625"/>
+    <col bestFit="true" customWidth="true" max="16" min="16" width="13.1640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
+    <row r="1" spans="1:19">
+      <c r="A1" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1201,7 +1214,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="17" thickBot="true">
       <c r="A2" s="5" t="s">
         <v>15</v>
       </c>
@@ -1226,7 +1239,9 @@
       <c r="H2" s="6">
         <v>5000</v>
       </c>
-      <c r="I2" s="6"/>
+      <c r="I2" s="6">
+        <v>-0.00</v>
+      </c>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
@@ -1244,7 +1259,7 @@
         <v>-35000</v>
       </c>
     </row>
-    <row r="3" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A3" s="5" t="s">
         <v>16</v>
       </c>
@@ -1269,7 +1284,9 @@
       <c r="H3" s="6">
         <v>542</v>
       </c>
-      <c r="I3" s="6"/>
+      <c r="I3" s="6">
+        <v>542.00</v>
+      </c>
       <c r="J3" s="6"/>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
@@ -1287,7 +1304,7 @@
         <v>-3794</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A4" s="5" t="s">
         <v>17</v>
       </c>
@@ -1312,7 +1329,9 @@
       <c r="H4" s="9">
         <v>527.75</v>
       </c>
-      <c r="I4" s="6"/>
+      <c r="I4" s="6">
+        <v>527.75</v>
+      </c>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
@@ -1330,7 +1349,7 @@
         <v>-3748</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
@@ -1355,7 +1374,9 @@
       <c r="H5" s="9">
         <v>0</v>
       </c>
-      <c r="I5" s="6"/>
+      <c r="I5" s="6">
+        <v>-0.00</v>
+      </c>
       <c r="J5" s="6"/>
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
@@ -1373,7 +1394,7 @@
         <v>-2660.2</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A6" s="5" t="s">
         <v>19</v>
       </c>
@@ -1398,7 +1419,9 @@
       <c r="H6" s="6">
         <v>281.2</v>
       </c>
-      <c r="I6" s="6"/>
+      <c r="I6" s="6">
+        <v>281.20</v>
+      </c>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
@@ -1416,7 +1439,7 @@
         <v>-1788.4</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A7" s="5" t="s">
         <v>20</v>
       </c>
@@ -1441,7 +1464,9 @@
       <c r="H7" s="9">
         <v>158.69999999999999</v>
       </c>
-      <c r="I7" s="6"/>
+      <c r="I7" s="6">
+        <v>158.70</v>
+      </c>
       <c r="J7" s="6"/>
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
@@ -1459,7 +1484,7 @@
         <v>-1232.92</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A8" s="10" t="s">
         <v>21</v>
       </c>
@@ -1484,7 +1509,9 @@
       <c r="H8" s="6">
         <v>0</v>
       </c>
-      <c r="I8" s="6"/>
+      <c r="I8" s="6">
+        <v>-0.00</v>
+      </c>
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
@@ -1502,7 +1529,7 @@
         <v>-1000.1400000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A9" s="10" t="s">
         <v>22</v>
       </c>
@@ -1527,7 +1554,9 @@
       <c r="H9" s="9">
         <v>9</v>
       </c>
-      <c r="I9" s="9"/>
+      <c r="I9" s="9">
+        <v>9.00</v>
+      </c>
       <c r="J9" s="9"/>
       <c r="K9" s="6"/>
       <c r="L9" s="6"/>
@@ -1545,7 +1574,7 @@
         <v>-72</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A10" s="12" t="s">
         <v>23</v>
       </c>
@@ -1570,7 +1599,9 @@
       <c r="H10" s="13">
         <v>0</v>
       </c>
-      <c r="I10" s="13"/>
+      <c r="I10" s="13">
+        <v>-0.00</v>
+      </c>
       <c r="J10" s="13"/>
       <c r="K10" s="13"/>
       <c r="L10" s="13"/>
@@ -1588,7 +1619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="17" thickBot="true">
       <c r="A11" s="16" t="s">
         <v>24</v>
       </c>
@@ -1633,7 +1664,7 @@
         <v>-9340.14</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A12" s="18" t="s">
         <v>25</v>
       </c>
@@ -1659,7 +1690,9 @@
       <c r="H12" s="17">
         <v>0</v>
       </c>
-      <c r="I12" s="19"/>
+      <c r="I12" s="19">
+        <v>390.00</v>
+      </c>
       <c r="J12" s="19"/>
       <c r="K12" s="19"/>
       <c r="L12" s="19"/>
@@ -1677,7 +1710,7 @@
         <v>-8939.4500000000007</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A13" s="18" t="s">
         <v>26</v>
       </c>
@@ -1722,7 +1755,7 @@
         <v>-5920.39</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A14" s="18" t="s">
         <v>27</v>
       </c>
@@ -1748,7 +1781,7 @@
         <v>582</v>
       </c>
       <c r="I14" s="17">
-        <v>582</v>
+        <v>582.00</v>
       </c>
       <c r="J14" s="17"/>
       <c r="K14" s="17"/>
@@ -1767,7 +1800,7 @@
         <v>-4799.97</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A15" s="18" t="s">
         <v>28</v>
       </c>
@@ -1797,7 +1830,9 @@
       <c r="H15" s="19">
         <v>390</v>
       </c>
-      <c r="I15" s="19"/>
+      <c r="I15" s="19">
+        <v>5486.98</v>
+      </c>
       <c r="J15" s="19"/>
       <c r="K15" s="17"/>
       <c r="L15" s="17"/>
@@ -1815,7 +1850,7 @@
         <v>-2428.13</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="18" thickTop="true" thickBot="true">
       <c r="A16" s="18" t="s">
         <v>29</v>
       </c>
@@ -1840,7 +1875,9 @@
       <c r="H16" s="19">
         <v>0</v>
       </c>
-      <c r="I16" s="19"/>
+      <c r="I16" s="19">
+        <v>-0.00</v>
+      </c>
       <c r="J16" s="19"/>
       <c r="K16" s="17"/>
       <c r="L16" s="17"/>
@@ -1858,7 +1895,7 @@
         <v>-1917.2099999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" ht="18" thickTop="true" thickBot="true">
       <c r="A17" s="18" t="s">
         <v>30</v>
       </c>
@@ -1883,7 +1920,9 @@
       <c r="H17" s="19">
         <v>0</v>
       </c>
-      <c r="I17" s="19"/>
+      <c r="I17" s="19">
+        <v>-0.00</v>
+      </c>
       <c r="J17" s="19"/>
       <c r="K17" s="17"/>
       <c r="L17" s="17"/>
@@ -1901,7 +1940,7 @@
         <v>-1413</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="18" thickTop="true" thickBot="true">
       <c r="A18" s="18" t="s">
         <v>31</v>
       </c>
@@ -1926,7 +1965,9 @@
       <c r="H18" s="17">
         <v>0</v>
       </c>
-      <c r="I18" s="17"/>
+      <c r="I18" s="17">
+        <v>-0.00</v>
+      </c>
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
       <c r="L18" s="17"/>
@@ -1944,7 +1985,7 @@
         <v>-260.52999999999997</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" ht="18" thickTop="true" thickBot="true">
       <c r="A19" s="18" t="s">
         <v>32</v>
       </c>
@@ -1969,7 +2010,9 @@
       <c r="H19" s="17">
         <v>0</v>
       </c>
-      <c r="I19" s="17"/>
+      <c r="I19" s="17">
+        <v>-0.00</v>
+      </c>
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
       <c r="L19" s="17"/>
@@ -1987,7 +2030,7 @@
         <v>-200</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" ht="18" thickTop="true" thickBot="true">
       <c r="A20" s="18" t="s">
         <v>33</v>
       </c>
@@ -2012,7 +2055,9 @@
       <c r="H20" s="17">
         <v>0</v>
       </c>
-      <c r="I20" s="17"/>
+      <c r="I20" s="17">
+        <v>-0.00</v>
+      </c>
       <c r="J20" s="17"/>
       <c r="K20" s="17"/>
       <c r="L20" s="17"/>
@@ -2030,7 +2075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:16" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="17" thickTop="true">
       <c r="A21" s="20" t="s">
         <v>34</v>
       </c>
@@ -2050,7 +2095,7 @@
       <c r="O21" s="22"/>
       <c r="P21" s="23"/>
     </row>
-    <row r="22" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" ht="17" thickBot="true">
       <c r="A22" s="24" t="s">
         <v>35</v>
       </c>
@@ -2081,7 +2126,9 @@
         <f>28889.9+386</f>
         <v>29275.9</v>
       </c>
-      <c r="I22" s="25"/>
+      <c r="I22" s="25">
+        <v>-0.00</v>
+      </c>
       <c r="J22" s="25"/>
       <c r="K22" s="25"/>
       <c r="L22" s="25"/>
@@ -2099,7 +2146,7 @@
         <v>199898.41999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:16" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" ht="18" thickTop="true" thickBot="true">
       <c r="A23" s="26" t="s">
         <v>27</v>
       </c>
@@ -2143,7 +2190,7 @@
         <v>2091</v>
       </c>
     </row>
-    <row r="24" spans="1:16" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="18" thickTop="true" thickBot="true">
       <c r="A24" s="26" t="s">
         <v>28</v>
       </c>
@@ -2188,7 +2235,7 @@
         <v>4348.2</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="17" thickTop="true">
       <c r="A25" s="29" t="s">
         <v>36</v>
       </c>
@@ -2208,7 +2255,7 @@
       <c r="O25" s="22"/>
       <c r="P25" s="23"/>
     </row>
-    <row r="26" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" ht="17" thickBot="true">
       <c r="A26" s="31" t="s">
         <v>37</v>
       </c>
@@ -2233,7 +2280,9 @@
       <c r="H26" s="32">
         <v>25000</v>
       </c>
-      <c r="I26" s="32"/>
+      <c r="I26" s="32">
+        <v>-0.00</v>
+      </c>
       <c r="J26" s="32"/>
       <c r="K26" s="32"/>
       <c r="L26" s="32"/>
@@ -2251,7 +2300,7 @@
         <v>175000</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" ht="17" thickTop="true">
       <c r="A27" s="33" t="s">
         <v>38</v>
       </c>
@@ -2271,61 +2320,61 @@
       <c r="O27" s="22"/>
       <c r="P27" s="23"/>
     </row>
-    <row r="28" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="35" t="s">
+    <row r="28" spans="1:16" ht="17" thickBot="true">
+      <c r="A28" s="41" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="36">
+      <c r="B28" s="35">
         <f t="shared" ref="B28:M28" si="3">(SUM(B2:B20)*-1)</f>
         <v>-12119.17</v>
       </c>
-      <c r="C28" s="36">
+      <c r="C28" s="35">
         <f t="shared" si="3"/>
         <v>-15247.02</v>
       </c>
-      <c r="D28" s="36">
+      <c r="D28" s="35">
         <f t="shared" si="3"/>
         <v>-9410.4700000000012</v>
       </c>
-      <c r="E28" s="36">
+      <c r="E28" s="35">
         <f t="shared" si="3"/>
         <v>-9752.7199999999993</v>
       </c>
-      <c r="F28" s="36">
+      <c r="F28" s="35">
         <f t="shared" si="3"/>
         <v>-12433.449999999999</v>
       </c>
-      <c r="G28" s="36">
+      <c r="G28" s="35">
         <f t="shared" si="3"/>
         <v>-17067.149999999994</v>
       </c>
-      <c r="H28" s="36">
+      <c r="H28" s="35">
         <f t="shared" si="3"/>
         <v>-8484.5</v>
       </c>
-      <c r="I28" s="36">
+      <c r="I28" s="35">
         <f t="shared" si="3"/>
-        <v>1575.85</v>
-      </c>
-      <c r="J28" s="36">
+        <v>0</v>
+      </c>
+      <c r="J28" s="35">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K28" s="36">
+      <c r="K28" s="35">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="L28" s="36">
+      <c r="L28" s="35">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="M28" s="36">
+      <c r="M28" s="35">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="N28" s="7">
         <f>AVERAGEIF(B28:M28,"&lt;&gt;0")</f>
-        <v>-10367.328749999999</v>
+        <v>-12073.497142857143</v>
       </c>
       <c r="O28" s="7">
         <f>MEDIAN(B28:M28)</f>
@@ -2333,58 +2382,58 @@
       </c>
       <c r="P28" s="8">
         <f>SUM(B28:M28)</f>
-        <v>-82938.62999999999</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="37" t="s">
+        <v>-84514.48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="18" thickTop="true" thickBot="true">
+      <c r="A29" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B29" s="38">
+      <c r="B29" s="36">
         <f t="shared" ref="B29:M29" si="4">SUM(B22:B24)</f>
         <v>27398</v>
       </c>
-      <c r="C29" s="38">
+      <c r="C29" s="36">
         <f t="shared" si="4"/>
         <v>27871</v>
       </c>
-      <c r="D29" s="38">
+      <c r="D29" s="36">
         <f t="shared" si="4"/>
         <v>27685.439999999999</v>
       </c>
-      <c r="E29" s="38">
+      <c r="E29" s="36">
         <f t="shared" si="4"/>
         <v>30001</v>
       </c>
-      <c r="F29" s="38">
+      <c r="F29" s="36">
         <f t="shared" si="4"/>
         <v>32575.02</v>
       </c>
-      <c r="G29" s="38">
+      <c r="G29" s="36">
         <f t="shared" si="4"/>
         <v>31531.26</v>
       </c>
-      <c r="H29" s="38">
+      <c r="H29" s="36">
         <f t="shared" si="4"/>
         <v>29275.9</v>
       </c>
-      <c r="I29" s="38">
+      <c r="I29" s="36">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J29" s="38">
+      <c r="J29" s="36">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="K29" s="38">
+      <c r="K29" s="36">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="L29" s="38">
+      <c r="L29" s="36">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="M29" s="38">
+      <c r="M29" s="36">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -2401,138 +2450,139 @@
         <v>206337.62</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A30" s="35" t="s">
+    <row r="30" spans="1:16">
+      <c r="A30" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="B30" s="36">
+      <c r="B30" s="35">
         <f t="shared" ref="B30:M30" si="5">SUM(B28,B29) - B26</f>
         <v>-9721.17</v>
       </c>
-      <c r="C30" s="36">
+      <c r="C30" s="35">
         <f t="shared" si="5"/>
         <v>-12376.02</v>
       </c>
-      <c r="D30" s="36">
+      <c r="D30" s="35">
         <f t="shared" si="5"/>
         <v>-6725.0300000000025</v>
       </c>
-      <c r="E30" s="36">
+      <c r="E30" s="35">
         <f t="shared" si="5"/>
         <v>-4751.7200000000012</v>
       </c>
-      <c r="F30" s="36">
+      <c r="F30" s="35">
         <f t="shared" si="5"/>
         <v>-4858.43</v>
       </c>
-      <c r="G30" s="36">
+      <c r="G30" s="35">
         <f t="shared" si="5"/>
         <v>-10535.889999999996</v>
       </c>
-      <c r="H30" s="36">
+      <c r="H30" s="35">
         <f t="shared" si="5"/>
         <v>-4208.5999999999985</v>
       </c>
-      <c r="I30" s="36">
+      <c r="I30" s="35">
         <f t="shared" si="5"/>
-        <v>1575.85</v>
-      </c>
-      <c r="J30" s="36">
+        <v>0</v>
+      </c>
+      <c r="J30" s="35">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="K30" s="36">
+      <c r="K30" s="35">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="L30" s="36">
+      <c r="L30" s="35">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="M30" s="36">
+      <c r="M30" s="35">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N30" s="39">
+      <c r="N30" s="37">
         <f>AVERAGEIF(B30:M30,"&lt;&gt;0")</f>
-        <v>-6450.1262499999993</v>
-      </c>
-      <c r="O30" s="39">
+        <v>-7596.6942857142849</v>
+      </c>
+      <c r="O30" s="37">
         <f>MEDIAN(B30:M30)</f>
         <v>-4480.16</v>
       </c>
-      <c r="P30" s="40">
+      <c r="P30" s="38">
         <f>SUM(B30:M30)</f>
-        <v>-51601.009999999995</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="41" t="s">
+        <v>-53176.859999999993</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="17" thickBot="true">
+      <c r="A31" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="B31" s="42">
+      <c r="B31" s="39">
         <f t="shared" ref="B31:M31" si="6">SUM(B28,B29)</f>
         <v>15278.83</v>
       </c>
-      <c r="C31" s="42">
+      <c r="C31" s="39">
         <f t="shared" si="6"/>
         <v>12623.98</v>
       </c>
-      <c r="D31" s="42">
+      <c r="D31" s="39">
         <f t="shared" si="6"/>
         <v>18274.969999999998</v>
       </c>
-      <c r="E31" s="42">
+      <c r="E31" s="39">
         <f t="shared" si="6"/>
         <v>20248.28</v>
       </c>
-      <c r="F31" s="42">
+      <c r="F31" s="39">
         <f t="shared" si="6"/>
         <v>20141.57</v>
       </c>
-      <c r="G31" s="42">
+      <c r="G31" s="39">
         <f t="shared" si="6"/>
         <v>14464.110000000004</v>
       </c>
-      <c r="H31" s="42">
+      <c r="H31" s="39">
         <f t="shared" si="6"/>
         <v>20791.400000000001</v>
       </c>
-      <c r="I31" s="42">
+      <c r="I31" s="39">
         <f t="shared" si="6"/>
-        <v>1575.85</v>
-      </c>
-      <c r="J31" s="42">
+        <v>0</v>
+      </c>
+      <c r="J31" s="39">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="K31" s="42">
+      <c r="K31" s="39">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="L31" s="42">
+      <c r="L31" s="39">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="M31" s="42">
+      <c r="M31" s="39">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="N31" s="14">
         <f>AVERAGEIF(B31:M31,"&lt;&gt;0")</f>
-        <v>15424.873750000002</v>
+        <v>17403.305714285718</v>
       </c>
       <c r="O31" s="14">
         <f>MEDIAN(B31:M31)</f>
         <v>13544.045000000002</v>
       </c>
-      <c r="P31" s="43">
+      <c r="P31" s="40">
         <f>SUM(B31:M31)</f>
-        <v>123398.99000000002</v>
+        <v>121823.14000000001</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup horizontalDpi="0" orientation="portrait" paperSize="9" verticalDpi="0"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>